<commit_message>
Update dataset_statistics.xlsx with revised data
</commit_message>
<xml_diff>
--- a/dataset_statistics.xlsx
+++ b/dataset_statistics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Datasets\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA57F94-6CC5-42A0-B201-340EB0B38CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3787CB0-F87E-488C-9C04-D70C909A2536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -502,10 +502,10 @@
         <v>1275</v>
       </c>
       <c r="D5" s="3">
-        <v>799</v>
+        <v>957</v>
       </c>
       <c r="E5" s="3">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="F5" s="3">
         <v>10</v>
@@ -525,16 +525,16 @@
         <v>4663</v>
       </c>
       <c r="D6" s="4">
-        <v>4618</v>
+        <v>4661</v>
       </c>
       <c r="E6" s="4">
-        <v>2849</v>
+        <v>3256</v>
       </c>
       <c r="F6" s="4">
-        <v>1414</v>
+        <v>1212</v>
       </c>
       <c r="G6" s="3">
-        <v>45</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -557,7 +557,7 @@
         <v>1368</v>
       </c>
       <c r="G7" s="4">
-        <v>1023</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -594,16 +594,16 @@
         <v>6875</v>
       </c>
       <c r="D9" s="4">
-        <v>5197</v>
+        <v>4975</v>
       </c>
       <c r="E9" s="4">
-        <v>1282</v>
+        <v>1271</v>
       </c>
       <c r="F9" s="3">
-        <v>529</v>
+        <v>509</v>
       </c>
       <c r="G9" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -623,10 +623,10 @@
         <v>6756</v>
       </c>
       <c r="F10" s="4">
-        <v>5027</v>
+        <v>4868</v>
       </c>
       <c r="G10" s="4">
-        <v>2799</v>
+        <v>2866</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -649,7 +649,7 @@
         <v>740</v>
       </c>
       <c r="G11" s="3">
-        <v>740</v>
+        <v>356</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -669,10 +669,10 @@
         <v>2657</v>
       </c>
       <c r="F12" s="3">
-        <v>652</v>
+        <v>864</v>
       </c>
       <c r="G12" s="3">
-        <v>164</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -692,10 +692,10 @@
         <v>1941</v>
       </c>
       <c r="F13" s="4">
-        <v>1845</v>
+        <v>1907</v>
       </c>
       <c r="G13" s="4">
-        <v>1696</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -712,13 +712,13 @@
         <v>2080</v>
       </c>
       <c r="E14" s="4">
-        <v>1470</v>
+        <v>1609</v>
       </c>
       <c r="F14" s="4">
-        <v>1093</v>
+        <v>1292</v>
       </c>
       <c r="G14" s="3">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -741,7 +741,7 @@
         <v>7662</v>
       </c>
       <c r="G15" s="4">
-        <v>4278</v>
+        <v>3921</v>
       </c>
     </row>
   </sheetData>

</xml_diff>